<commit_message>
Add test email rajsonisharma385@gmail.com to test_guests.xlsx
</commit_message>
<xml_diff>
--- a/test_guests.xlsx
+++ b/test_guests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -570,6 +570,28 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Raj Soni Sharma</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>rajsonisharma385@gmail.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ROLL007</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>9876543216</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>